<commit_message>
feat(branch): run-003 discovery, test design, and SHAFT automation for Search/Actions + Update Branch
Adds the run-003 artifacts for US-8599 (Search & Actions) and US-8606
(Update Branch):

- Discovery snapshots for the Search Branch and Update Branch screens with
  supporting evidence, plus FINDING-012..015 (missing State column, Branch
  Email Password returned to the client, Active/Inactive status not shown,
  City filter is multi-select).
- Regenerated test design (cases, traceability matrix, coverage report) and
  refreshed Stage 4A automation reports for the extended scope.
- SHAFT suite grows Search/Update/Actions coverage: AbstractBaseTest, the
  BasePage/SearchBranchPage/UpdateBranchPage page objects, the corresponding
  test classes, and BranchProvisioner for seeding records.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/platform_core_data/modules/branch/test_design/TestCases_Branch.xlsx
+++ b/platform_core_data/modules/branch/test_design/TestCases_Branch.xlsx
@@ -60,7 +60,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:L40"/>
+  <dimension ref="A1:L82"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -2473,6 +2473,2462 @@
         </is>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-BR-040</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Search Branch by Branch Code returns the matching record</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that searching by a known Branch Code returns that branch.</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">User is logged in as Super Admin and has opened Admin → Branch.</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">| Field | Value |
+|---|---|
+| Branch Code | BRN2 |</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Enter the Test Data value in the **Branch code** field. | 2. Click **Search**.</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The grid returns the branch whose Code is `BRN2`.</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Positive, Smoke</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-BR-041</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Search Branch by Branch Name returns the matching record</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that searching by Branch Name returns branches whose name matches.</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">User is logged in as Super Admin and has opened Admin → Branch.</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">| Field | Value |
+|---|---|
+| Branch Name | Emirates NDC |</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Enter the Test Data value in the **Branch name** field. | 2. Click **Search**.</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The grid returns the branch named `Emirates NDC`.</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Positive, Smoke</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-BR-042</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Search with no criteria returns the default Active result set</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that searching without entering any criteria returns all Active branches.</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">User is logged in as Super Admin and has opened Admin → Branch.</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Leave every filter at its default. | 2. Click **Search**.</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The grid returns results and the count text states the total number of Active branches. No validation error is shown.</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Positive</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-BR-043</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Search with non-matching criteria shows the empty-state message</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that a search returning no records displays the platform's empty-state message rather than a blank grid.</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">User is logged in as Super Admin and has opened Admin → Branch.</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">| Field | Value |
+|---|---|
+| Branch Code | ZZZZQQ9 |</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Enter the Test Data value in the **Branch code** field. | 2. Click **Search**.</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The message `No data has been found!` is displayed and the grid shows no rows.</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Negative-InvalidInputs, Regression</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-BR-044</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Status filter defaults to Active on page load</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that the Status radio group has Active pre-selected when the screen loads.</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">User is logged in as Super Admin.</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Open Admin → Branch. | 2. Read the Status radio group without changing it.</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">**Active** is selected. **Inactive** and **Both** are not selected.</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Positive, BusinessRule</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Rejected</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-BR-045</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Status filter returns only records matching the selected status</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that each Status option returns only branches in that state, and that Both returns the union.</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">User is logged in as Super Admin and has opened Admin → Branch.</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">| Status selected |
+|---|
+| Active |
+| Inactive |
+| Both |</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Select the Status option under test. | 2. Click **Search**. | 3. Record the total from the result count text. | 4. Repeat steps 1–3 for each option in Test Data.</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Each search returns a result set, and the Both total equals the Active total plus the Inactive total.</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Positive, BusinessRule, Regression</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Discovery observed 491 Active + 125 Inactive = 616 Both. Compare the totals to each other rather than to those fixed numbers — the environment is shared and counts change.</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-BR-046</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">State filter stays disabled until a Country is selected</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that the State filter becomes usable only after a Country is chosen.</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">User is logged in as Super Admin and has opened Admin → Branch.</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Observe the **State** filter before selecting a Country. | 2. Select **Egypt** in the **Country** filter. | 3. Observe the **State** filter again.</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">State is disabled at step 1 and enabled at step 3, listing states belonging to Egypt.</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Positive, BusinessRule</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-BR-047</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">City filter stays disabled until a State is selected</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that the City filter becomes usable only after a State is chosen.</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">User is logged in as Super Admin and has opened Admin → Branch, with Country set to Egypt.</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Observe the **City** filter before selecting a State. | 2. Select any State. | 3. Observe the **City** filter again.</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">City is disabled at step 1 and enabled at step 3, listing cities belonging to the selected State.</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Positive, BusinessRule</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Rejected</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-BR-048</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Branch Code filter accepts alphanumeric input</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that the Branch Code filter accepts letters and digits.</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">User is logged in as Super Admin and has opened Admin → Branch.</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">| Field | Value |
+|---|---|
+| Branch Code | BRN262 |</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Enter the Test Data value in the **Branch code** field. | 2. Click **Search**.</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The value is accepted with no validation error and the search executes.</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P3</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Positive</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Rejected</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-BR-049</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Branch Name filter accepts alphabetic and special characters</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that the Branch Name filter accepts letters and special characters as the acceptance criteria state.</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">User is logged in as Super Admin and has opened Admin → Branch.</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">| Field | Value |
+|---|---|
+| Branch Name | Test-Branch &amp; Co. |</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Enter the Test Data value in the **Branch name** field. | 2. Click **Search**.</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The value is accepted with no validation error and the search executes.</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P3</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Positive</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Rejected</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-BR-050</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Branch Name filter handles Unicode input without error</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that non-ASCII input in the Branch Name filter is handled without an unhandled error.</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">User is logged in as Super Admin and has opened Admin → Branch.</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">| Field | Value |
+|---|---|
+| Branch Name | القاهرة 東京 🏢 |</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Enter the Test Data value in the **Branch name** field. | 2. Click **Search**.</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The search completes. Either matching records or `No data has been found!` is displayed. No unhandled error, blank page, or server error appears.</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P3</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Negative-Unicode</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Rejected</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-BR-051</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Search filters handle security-payload-shaped input safely</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that payload-shaped strings in the search filters are treated as literal text.</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">User is logged in as Super Admin and has opened Admin → Branch.</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">| Field | Value |
+|---|---|
+| Branch Name | `&lt;script&gt;alert(1)&lt;/script&gt;` |
+| Branch Code | `' OR '1'='1` |</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Enter the Branch Name value and click **Search**. | 2. Clear the field, enter the Branch Code value and click **Search**.</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Each search completes and returns either matching records or `No data has been found!`. No script executes, no database error is exposed, and no unfiltered result set is returned.</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Negative-SecurityInputs</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Input-handling probe only — observe the response, never attempt to exploit.</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Rejected</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-BR-052</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Results grid displays all specified columns</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that the results grid shows every column the acceptance criteria require.</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">User is logged in as Super Admin and has opened Admin → Branch.</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Click **Search**. | 2. Read the grid's header row.</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The grid displays Branch Code, Branch Name, Country Name, **State**, City, Approval Status, and Actions columns.</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Regression</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">This asserts the corrected behaviour. Discovery confirmed the State column is currently absent (FINDING-012) — this case is expected to fail until that is fixed or the requirement is formally changed.</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-BR-053</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approval Status column reflects each record's approval state</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that the Approval Status column shows the record's current approval state.</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">User is logged in as Super Admin and has opened Admin → Branch.</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Select Status **Both**. | 2. Click **Search**. | 3. Read the Approval Status value on each row.</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Every row shows one of `Approved`, `Pending for approval`, or `Rejected`. No row shows a blank Approval Status.</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Positive</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Rejected</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-BR-054</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Row action icons match the record's approval state</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that each row offers only the actions valid for its approval state.</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">User is logged in as Super Admin and has opened Admin → Branch, with Status set to Both and results displayed.</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">| Approval Status | Expected icons |
+|---|---|
+| Approved | edit pen, thumbs-down |
+| Pending for approval | edit pen, thumbs-up, thumbs-down |
+| Rejected | edit pen, thumbs-up |</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Locate a row for each Approval Status in the Test Data. | 2. Read the icons in that row's Actions column.</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Each row shows exactly the icons listed for its Approval Status — a record never offers a transition to the state it is already in.</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Positive</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Pending and Rejected rows may not appear on page 1; page through the results or search for a known record to find one.</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-BR-055</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Edit pen opens Update Branch with the record's details pre-filled</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that the edit pen navigates to Update Branch showing the selected branch's stored values.</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">User is logged in as Super Admin and has opened Admin → Branch, with results displayed.</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Note the Code, Branch Name, Country Name and City shown on a chosen row. | 2. Click that row's edit pen icon. | 3. Wait until the Branch Name field shows a value. | 4. Compare the form's Name, Country, State and City against the values noted in step 1.</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The Update Branch screen opens for the selected branch, and its Name, Country, State and City match the values shown in the grid row.</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Scenario, Positive, Smoke</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Step 3 matters — wait for a field to actually populate before comparing. Reading the form on a fixed delay produced a false "form is empty" result twice during Discovery.</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-BR-056</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approve a Pending branch from the results grid</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that the thumbs-up action approves a branch awaiting approval.</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">User is logged in as Super Admin. A branch created by this run exists with Approval Status `Pending for approval`, and its Branch Code has been recorded.</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">| Field | Value |
+|---|---|
+| Branch Code | the code of the branch this run created |</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Search for the recorded Branch Code. | 2. Confirm the row's Approval Status reads `Pending for approval`. | 3. Click that row's thumbs-up icon. | 4. Complete any prompt that appears. | 5. Search for the same Branch Code again.</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The branch's Approval Status changes to `Approved`, and its row now offers the edit pen and thumbs-down only.</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Scenario, Positive, SelfCreatedRecord</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Act only on a branch this run created. Record its Branch Code before acting — acting on a pre-existing branch is not authorised for this run.</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-BR-057</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Reject a Pending branch from the results grid</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that the thumbs-down action rejects a branch awaiting approval.</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">User is logged in as Super Admin. A second branch created by this run exists with Approval Status `Pending for approval`, and its Branch Code has been recorded.</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">| Field | Value |
+|---|---|
+| Branch Code | the code of a second branch this run created |</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Search for the recorded Branch Code. | 2. Confirm the row's Approval Status reads `Pending for approval`. | 3. Click that row's thumbs-down icon. | 4. Complete any prompt that appears. | 5. Search for the same Branch Code again.</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The branch's Approval Status changes to `Rejected`, and its row now offers the edit pen and thumbs-up only.</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Scenario, Positive, SelfCreatedRecord</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Use a different self-created branch from TC-BR-056 so each case starts from a Pending record.</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-BR-058</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approve and Reject capture a Remarks entry</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that approving or rejecting a branch records a free-text Remarks reason.</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">User is logged in as Super Admin. A branch created by this run exists with Approval Status `Pending for approval`.</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">| Field | Value |
+|---|---|
+| Remarks | Approved by QA run-003 |</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Search for the self-created branch. | 2. Click the thumbs-up icon. | 3. Observe whether a Remarks entry is requested. | 4. If it is, enter the Test Data value and confirm.</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">A Remarks entry is requested before the approval completes, the entered text is accepted, and the approval succeeds.</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Positive, SelfCreatedRecord</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Discovery could not establish whether the grid-level action prompts for Remarks — the Update screen has a mandatory Remarks field, but the grid path was never exercised. If no prompt appears, record that as the observed result rather than a pass.</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-BR-059</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Same account attempts to approve the branch it created</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify whether the account that created a branch is permitted to approve it.</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">User is logged in as Super Admin and has just created a branch with this same account, leaving it `Pending for approval`. Its Branch Code has been recorded.</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Search for the branch this account just created. | 2. Click that row's thumbs-up icon. | 3. Observe the outcome. | 4. Search for the branch again and read its Approval Status.</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Record which of the following occurs: the approval succeeds and the status becomes `Approved`, or the action is blocked with a message. Capture the exact message if one appears.</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Security, SelfCreatedRecord, AssumptionBased</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Assumption-based — the requirement that a maker cannot approve their own change is inferred, not asserted, in the source material. Either outcome is a valid result. Because this run has only one account, a blocked result must be reported as "appears blocked" — there is no second account to prove that approval by a different user would have succeeded.</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Rejected</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-BR-060</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Navigate to the next page of results</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that the next-page control advances through the result set.</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">User is logged in as Super Admin, with a search returning more rows than one page.</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Note the Branch Codes shown on page 1. | 2. Click the next-page control. | 3. Read the Branch Codes now shown.</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">A different set of records is displayed, and none of the page 1 codes reappear.</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Positive</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-BR-061</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Navigate to the last page of results</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that the last-page control jumps to the final page of results.</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">User is logged in as Super Admin, with a search returning several pages.</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Click the **Last** control. | 2. Read the page indicator and the rows displayed.</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The final page is displayed with at least one row, and no further next-page navigation is offered.</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P3</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Positive</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-BR-062</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Pagination preserves the active status filter</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that changing pages does not reset the selected Status filter.</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">User is logged in as Super Admin and has opened Admin → Branch.</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Select Status **Both** and click **Search**. | 2. Note the total shown in the result count text. | 3. Navigate forward two pages. | 4. Read the Status radio group and the result count text.</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">**Both** is still selected and the total is unchanged from step 2.</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Positive, Regression</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Rejected</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-BR-063</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Result count text reflects the filtered total</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that the result count text states the total for the applied filter.</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">User is logged in as Super Admin and has opened Admin → Branch.</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Select Status **Active** and click **Search**; read the count text. | 2. Select Status **Inactive** and click **Search**; read the count text.</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The count text is displayed in each case and its stated total changes between the two searches.</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P3</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Positive</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Rejected</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-BR-064</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">A record on a later page is findable by direct search</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that a branch not on page 1 can still be retrieved by searching for it.</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">User is logged in as Super Admin and has opened Admin → Branch.</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Select Status **Both**, click **Search**, and page forward until a row is visible that was not on page 1. | 2. Note that row's Branch Code. | 3. Return to Admin → Branch and enter the noted code in the **Branch code** field. | 4. Click **Search**.</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The branch is returned on the first page of results.</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Positive</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Rejected</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-BR-065</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Update Branch pre-fills every stored value</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that opening a branch for update shows all of its stored values.</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">User is logged in as Super Admin and has opened a branch via the edit pen.</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Wait until the Branch Name field shows a value. | 2. Read Operating Country, Name, Country, State, City, Post Office Box, Email ID, Credit Limit, Top Up Limit and Outstanding Threshold.</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Every field listed in step 2 shows the branch's stored value. No field that holds data is blank, and neither State nor City shows an unselected placeholder.</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Scenario, Positive, Smoke</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Wait for a field to populate before reading — a fixed delay produced a false "form is empty" result twice during Discovery.</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-BR-066</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Update a branch and submit it for approval</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that an edited branch can be submitted for approval and returns to a pending state.</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">User is logged in as Super Admin. A branch created by this run is open on the Update Branch screen.</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">| Field | Value |
+|---|---|
+| Address 1 | Updated by QA run-003 |
+| Remarks | Address corrected |</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Change **Address 1** to the Test Data value. | 2. Enter the Remarks value. | 3. Click **Send For Approval**. | 4. Search for the branch on Admin → Branch.</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The update is saved, a success confirmation is shown, and the branch's Approval Status reads `Pending for approval`.</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Scenario, Positive, SelfCreatedRecord</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The button is labelled `Send For Approval`, not "Submit for Approval" — see FINDING-011. Act only on a branch this run created.</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-BR-067</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Remarks is mandatory before any Update action</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that an Update action is blocked when Remarks is empty.</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">User is logged in as Super Admin. A branch created by this run is open on the Update Branch screen.</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Change **Address 1** to any valid value. | 2. Leave **Remarks** empty. | 3. Click **Send For Approval**.</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Submission is blocked and a required-field validation message is shown for Remarks.</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Negative-EmptyValues, SelfCreatedRecord</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-BR-068</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Cancel discards unsaved changes on Update Branch</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that Cancel exits without saving edits.</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">User is logged in as Super Admin. A branch created by this run is open on the Update Branch screen.</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Change **Address 1** to a new value. | 2. Click **Cancel**. | 3. Re-open the same branch via the edit pen and wait for the form to populate. | 4. Read **Address 1**.</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Address 1 shows its original value; the change made in step 1 was not saved.</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Positive, SelfCreatedRecord</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-BR-069</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approve a branch update request from the Update screen</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that a pending branch update can be approved from the Update Branch screen.</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">User is logged in as Super Admin. A branch created by this run has a pending update and is open on the Update Branch screen.</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">| Field | Value |
+|---|---|
+| Remarks | Update approved by QA run-003 |</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Enter the Remarks value. | 2. Click **Approve**. | 3. Search for the branch on Admin → Branch.</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">A success confirmation is shown and the branch's Approval Status reads `Approved`.</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Scenario, Positive, SelfCreatedRecord</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-BR-070</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Reject a branch update request from the Update screen</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that a pending branch update can be rejected from the Update Branch screen.</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">User is logged in as Super Admin. A second branch created by this run has a pending update and is open on the Update Branch screen.</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">| Field | Value |
+|---|---|
+| Remarks | Update rejected by QA run-003 |</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Enter the Remarks value. | 2. Click **Reject**. | 3. Search for the branch on Admin → Branch.</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">A confirmation is shown and the branch's Approval Status reads `Rejected`.</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Scenario, Positive, SelfCreatedRecord</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Rejected</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-BR-071</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Mandatory Update Branch fields block submission when cleared</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that clearing a mandatory field on Update blocks submission.</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">User is logged in as Super Admin. A branch created by this run is open on the Update Branch screen, with the form populated.</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">| Field Cleared |
+|---|
+| Name |
+| State |
+| City |
+| Address 1 |
+| Post Office Box |
+| Credit Limit |
+| Top Up Limit |
+| Credit Terms (Days) |</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Clear the one field under test. | 2. Enter a valid Remarks value. | 3. Click **Send For Approval**. | 4. Restore the field's original value and repeat steps 1–3 for each field in Test Data.</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">For each field cleared, submission is blocked and a required-field validation message is shown for that field.</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Negative-EmptyValues, SelfCreatedRecord</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Rejected</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-BR-072</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Post Office Box rejects a value exceeding 8 characters on Update</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that the Update screen enforces the 8-character limit on Post Office Box.</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">User is logged in as Super Admin. A branch created by this run is open on the Update Branch screen.</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">| Field | Value |
+|---|---|
+| Post Office Box | ABCD123456 |
+| Remarks | Boundary check |</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Replace **Post Office Box** with the 10-character Test Data value. | 2. Enter the Remarks value. | 3. Click **Send For Approval**.</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The field either truncates the entry to 8 characters or blocks submission with a length validation message.</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Negative-BoundaryValues, Regression, SelfCreatedRecord</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The Create screen accepts over-length values without enforcement (FINDING-002). This asserts the corrected behaviour on Update and is expected to fail if the same gap exists there.</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Rejected</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-BR-073</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Credit Limit rejects a value exceeding 15 characters on Update</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that the Update screen enforces the 15-character limit on Credit Limit.</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">User is logged in as Super Admin. A branch created by this run is open on the Update Branch screen.</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">| Field | Value |
+|---|---|
+| Credit Limit | 1234567890123456 |
+| Remarks | Boundary check |</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Replace **Credit Limit** with the 16-digit Test Data value. | 2. Enter the Remarks value. | 3. Click **Send For Approval**.</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The field either truncates the entry to 15 digits or blocks submission with a length validation message.</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Negative-BoundaryValues, Regression, SelfCreatedRecord</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Mirrors FINDING-003 on the Create screen. Asserts the corrected behaviour.</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Rejected</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-BR-074</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Warning Prompt must not exceed Credit Terms on Update</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that the cross-field rule between Warning Prompt and Credit Terms is enforced on Update.</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">User is logged in as Super Admin. A branch created by this run is open on the Update Branch screen.</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">| Field | Value |
+|---|---|
+| Credit Terms (Days) | 10 |
+| Warning Prompt (Days) | 20 |
+| Remarks | Cross-field check |</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Set **Credit Terms (Days)** to 10. | 2. Set **Warning Prompt (Days)** to 20. | 3. Enter the Remarks value. | 4. Click **Send For Approval**.</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Submission is blocked with a message stating the warning prompt days must not be greater than the credit terms days.</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Negative-InvalidInputs, SelfCreatedRecord</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">This rule is confirmed enforced on the Create screen; equal values are permitted there and only a greater value is rejected.</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Rejected</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-BR-075</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Reaching Percentage rejects a value above 100 on Update</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that Reaching Percentage cannot exceed 100 on the Update screen.</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">User is logged in as Super Admin. A branch created by this run is open on the Update Branch screen.</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">| Field | Value |
+|---|---|
+| Reaching Percentage | 101 |
+| Remarks | Boundary check |</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Set **Reaching Percentage** to 101. | 2. Enter the Remarks value. | 3. Click **Send For Approval**.</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Submission is blocked with a validation message indicating the percentage may not exceed 100.</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Negative-BoundaryValues, SelfCreatedRecord</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Rejected</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-BR-076</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Change Threshold lists child agencies before confirming</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that changing a branch threshold surfaces the child agencies affected before the change is confirmed.</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">User is logged in as Super Admin. A branch created by this run is open on the Update Branch screen.</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">| Field | Value |
+|---|---|
+| Outstanding Threshold | 50 |</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Change **Outstanding Threshold** to the Test Data value. | 2. Click **Change Threshold**. | 3. Read the confirmation popup.</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">A confirmation popup appears listing any child agencies holding a custom threshold, and offers the option to confirm or cancel before the change is applied.</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Scenario, Positive, SelfCreatedRecord, AssumptionBased</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Assumption-based — this flow was never exercised during Discovery. A branch created by this run will have no child agencies, so the popup may legitimately show an empty list; record what appears rather than treating an empty list as a failure.</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Rejected</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-BR-077</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Stored Branch Email Password is not recoverable from the Update form</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that a branch's stored email password is not returned to the browser when the Update screen loads.</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">User is logged in as Super Admin and has opened any branch via the edit pen.</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Wait until the form has populated. | 2. Inspect the **Email Password** field's underlying value using browser developer tools.</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The field holds no recoverable password value — it is empty, or contains only a placeholder that is not the stored password.</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Security, Regression</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Asserts the corrected behaviour. Discovery confirmed the stored password is currently returned and populated into this field (FINDING-013), so this case is expected to fail until that is fixed. **Never record the observed password value in a result, defect, or screenshot** — report only whether a recoverable value was present.</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Rejected</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-BR-078</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Exploratory — is Active/Inactive status discoverable from the grid?</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Determine whether an operator can tell an Active branch from an Inactive one in the results grid.</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">User is logged in as Super Admin and has opened Admin → Branch.</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Select Status **Both** and click **Search**. | 2. Attempt to determine, from the grid alone, which returned records are Active and which are Inactive. | 3. Note every column, icon, or styling cue that conveys it, if any.</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Confirm with the reviewer whether operating without an Active/Inactive indicator in the grid is acceptable, or whether the grid must expose that status as a column.</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Exploratory</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Exploratory pending a Product decision (FINDING-014). The acceptance criteria do not list an Active/Inactive column, but the platform-wide convention treats Status and Approval Status as distinct columns. Do not record a pass or fail — record the observation and the reviewer's decision.</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Rejected</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-BR-079</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Exploratory — does the City filter accept and apply multiple cities?</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Determine whether the City filter's multi-select capability works and is intended.</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">User is logged in as Super Admin and has opened Admin → Branch, with a Country and State selected.</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Open the **City** filter and attempt to select two or more cities. | 2. Click **Search**. | 3. Check whether the results include branches from every selected city.</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Confirm with the reviewer whether multi-city selection is intended behaviour, and if so, whether the acceptance criteria should be updated to describe a multi-select rather than a dropdown.</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P3</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Exploratory</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Exploratory pending a Product decision (FINDING-015). The control is built as a multi-select; the acceptance criteria specify a dropdown. Do not record a pass or fail.</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Rejected</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-BR-080</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Admin-role operator sees the same grid columns and row actions</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that an Admin-role operator sees the same Search Branch surface as a Super Admin.</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">An Admin-role account exists and its credentials are available.</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Log in as an Admin-role user. | 2. Open Admin → Branch and click **Search**. | 3. Compare the grid columns and the row action icons against those seen as Super Admin.</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Confirm whether the Admin role sees the same columns and the same row actions, and record any difference.</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P3</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Permissions, NotCovered-SingleAccountRun</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">**Not executable this run.** Only one account is available, and it holds Super Admin privileges while standing in for both actors — a privileged account cannot demonstrate an unprivileged view. Record as `Not Covered — Single-Account Run`, never as passed. Unblocked by provisioning an Admin-role credential.</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Rejected</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TC-BR-081</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Repeated failed login attempts lock the account</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Verify that the account lock rule triggers after repeated failed authentication attempts.</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">A dedicated, non-shared environment with a disposable account.</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">| Field | Value |
+|---|---|
+| Password | a deliberately incorrect value |</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1. Attempt to log in with a valid username and an incorrect password. | 2. Repeat until the documented lock threshold is exceeded. | 3. Attempt to log in with the correct password.</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">After the threshold is exceeded the account is locked and a lock message is shown; the correct password no longer grants access until the account is unlocked.</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">P3</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Atomic, Security, Deferred-RequiresDedicatedEnvironment</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">**Deferred — Requires Dedicated Environment.** Designed in full but not for execution on the shared staging environment: locking a shared account would block other teams, and the lock is not self-reversing. Execute only on an isolated environment with a disposable account.</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Approved</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Rejected</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>